<commit_message>
Add foundry FDE skill library and lean operating-model scenario
foundry/: five versioned agent skills (orchestrator, data profiling,
adapter mapping, GL reconciliation, validation pack), a customer pod
template run through the Workbench MCP ops profile, and a gate-record
schema with human-only approval.

business/: operating-model selector (standard FDE team vs lean agent
foundry) with lean delivery and cost inputs, an FDE capacity check row,
and the generator script for the workbook.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WXgVqEVUV2oamzUfYvRj6M
</commit_message>
<xml_diff>
--- a/business/rates-workbench-business-model.xlsx
+++ b/business/rates-workbench-business-model.xlsx
@@ -27,6 +27,18 @@
     <author>Unknown Author</author>
   </authors>
   <commentList>
+    <comment ref="C3" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Lean: agent pods do integration/validation drafting; one FDE supervises several banks in parallel</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="C5" authorId="0">
       <text>
         <r>
@@ -107,7 +119,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">1 month x 2 FDEs + validation support</t>
+          <t xml:space="preserve">Standard: 1 month x 2 FDEs + validation support. Lean: ~1 FDE-month supervising agents</t>
         </r>
       </text>
     </comment>
@@ -119,7 +131,19 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">First integrations take 2–3 months</t>
+          <t xml:space="preserve">First integrations take 2–3 months; skills are still being built</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C27" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Lean: upgrades/customization run by agents with gated review</t>
         </r>
       </text>
     </comment>
@@ -210,7 +234,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="158">
   <si>
     <t xml:space="preserve">Rates Workbench – business model assumptions</t>
   </si>
@@ -218,6 +242,9 @@
     <t xml:space="preserve">Blue = editable input; yellow = key lever. All $ in $M. Figures are illustrative judgment, not market data.</t>
   </si>
   <si>
+    <t xml:space="preserve">Operating model (1=Standard FDE team, 2=Lean agent foundry)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Scalar inputs</t>
   </si>
   <si>
@@ -281,6 +308,15 @@
     <t xml:space="preserve">Delivery effort</t>
   </si>
   <si>
+    <t xml:space="preserve">Standard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lean</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Active</t>
+  </si>
+  <si>
     <t xml:space="preserve">FDE-years per new Large bank</t>
   </si>
   <si>
@@ -383,6 +419,42 @@
     <t xml:space="preserve">Advisory enterprise licenses (base)</t>
   </si>
   <si>
+    <t xml:space="preserve">Core R&amp;D / quant heads – standard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sales heads – standard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Partner-enablement heads – standard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G&amp;A heads – standard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Non-personnel costs, $M – standard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lean agent-foundry inputs (used when C3 = 2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Core R&amp;D / quant heads – lean</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sales heads – lean</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Partner-enablement heads – lean</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G&amp;A heads – lean</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Non-personnel costs, $M – lean (incl. agent tokens/compute/security)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Active cost inputs (from operating model)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Core R&amp;D / quant heads</t>
   </si>
   <si>
@@ -398,7 +470,7 @@
     <t xml:space="preserve">Non-personnel costs, $M</t>
   </si>
   <si>
-    <t xml:space="preserve">Example: to test a slower ramp, set C5 to 1, or lower row 48–49 deal counts.</t>
+    <t xml:space="preserve">Example: set C3 to 1 for the standard FDE team, C5 to 1 for a slower ramp, or lower row 48–49 deal counts.</t>
   </si>
   <si>
     <t xml:space="preserve">Projections ($M unless noted) – scenario-driven</t>
@@ -531,6 +603,12 @@
   </si>
   <si>
     <t xml:space="preserve">Peak funding need (excl. Phase-0 and buffer)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New banks onboarded per FDE (capacity check)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One FDE supervising agent pods handles ~4–6 concurrent onboardings (~30–50 a year); above that, hire.</t>
   </si>
   <si>
     <t xml:space="preserve">Valuation – Year 5 exit and implied value today</t>
@@ -683,13 +761,6 @@
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
-      <sz val="11"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
       <sz val="11"/>
       <name val="Arial"/>
       <family val="0"/>
@@ -698,6 +769,13 @@
     <font>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -786,15 +864,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -802,7 +876,55 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -810,51 +932,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1114,10 +1192,10 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G61"/>
+  <dimension ref="A1:G76"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="2" style="0" width="12"/>
   </cols>
   <sheetData>
@@ -1131,49 +1209,57 @@
         <v>1</v>
       </c>
     </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>2</v>
+      </c>
+    </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="C4" s="3" t="s">
+      <c r="A4" s="5" t="s">
         <v>3</v>
       </c>
+      <c r="C4" s="5" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C5" s="5" t="n">
+      <c r="A5" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="4" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
-        <v>5</v>
+      <c r="A6" s="3" t="s">
+        <v>6</v>
       </c>
       <c r="C6" s="6" t="n">
         <v>0.5</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
-        <v>6</v>
+      <c r="A7" s="3" t="s">
+        <v>7</v>
       </c>
       <c r="C7" s="6" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
-        <v>7</v>
+      <c r="A8" s="3" t="s">
+        <v>8</v>
       </c>
       <c r="C8" s="6" t="n">
         <v>1.4</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
-        <v>8</v>
+      <c r="A9" s="3" t="s">
+        <v>9</v>
       </c>
       <c r="C9" s="7" t="n">
         <f aca="false">INDEX(C6:C8,C5)</f>
@@ -1181,527 +1267,578 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
-        <v>9</v>
+      <c r="A10" s="5" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
-        <v>10</v>
+      <c r="A11" s="3" t="s">
+        <v>11</v>
       </c>
       <c r="C11" s="8" t="n">
         <v>0.8</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
-        <v>11</v>
+      <c r="A12" s="3" t="s">
+        <v>12</v>
       </c>
       <c r="C12" s="8" t="n">
         <v>0.35</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
-        <v>12</v>
+      <c r="A13" s="3" t="s">
+        <v>13</v>
       </c>
       <c r="C13" s="9" t="n">
         <v>0.25</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="s">
-        <v>13</v>
+      <c r="A14" s="3" t="s">
+        <v>14</v>
       </c>
       <c r="C14" s="10" t="n">
         <v>0.8</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
-        <v>14</v>
+      <c r="A15" s="3" t="s">
+        <v>15</v>
       </c>
       <c r="C15" s="9" t="n">
         <v>0.25</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
-        <v>15</v>
+      <c r="A16" s="3" t="s">
+        <v>16</v>
       </c>
       <c r="C16" s="9" t="n">
         <v>0.15</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
-        <v>16</v>
+      <c r="A17" s="3" t="s">
+        <v>17</v>
       </c>
       <c r="C17" s="9" t="n">
         <v>0.15</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="s">
-        <v>17</v>
+      <c r="A18" s="3" t="s">
+        <v>18</v>
       </c>
       <c r="C18" s="10" t="n">
         <v>0.2</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="s">
-        <v>18</v>
+      <c r="A19" s="3" t="s">
+        <v>19</v>
       </c>
       <c r="C19" s="9" t="n">
         <v>0.15</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="s">
-        <v>19</v>
+      <c r="A20" s="3" t="s">
+        <v>20</v>
       </c>
       <c r="C20" s="9" t="n">
         <v>0.15</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="s">
-        <v>20</v>
+      <c r="A21" s="3" t="s">
+        <v>21</v>
       </c>
       <c r="C21" s="9" t="n">
         <v>0.075</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="s">
-        <v>21</v>
+      <c r="A22" s="3" t="s">
+        <v>22</v>
       </c>
       <c r="C22" s="9" t="n">
         <v>0.15</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="3" t="s">
-        <v>22</v>
+      <c r="A23" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4" t="s">
-        <v>23</v>
+      <c r="A24" s="3" t="s">
+        <v>27</v>
       </c>
       <c r="C24" s="11" t="n">
         <v>0.3</v>
       </c>
+      <c r="D24" s="11" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E24" s="12" t="n">
+        <f aca="false">IF($C$3=1,C24,D24)</f>
+        <v>0.1</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="C25" s="12" t="n">
+      <c r="A25" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C25" s="13" t="n">
         <v>0.25</v>
       </c>
+      <c r="D25" s="13" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="E25" s="12" t="n">
+        <f aca="false">IF($C$3=1,C25,D25)</f>
+        <v>0.08</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C26" s="12" t="n">
+      <c r="A26" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C26" s="13" t="n">
         <v>0.5</v>
       </c>
+      <c r="D26" s="13" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E26" s="12" t="n">
+        <f aca="false">IF($C$3=1,C26,D26)</f>
+        <v>0.25</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="C27" s="12" t="n">
+      <c r="A27" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C27" s="13" t="n">
         <v>0.25</v>
       </c>
+      <c r="D27" s="13" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E27" s="12" t="n">
+        <f aca="false">IF($C$3=1,C27,D27)</f>
+        <v>0.05</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C28" s="12" t="n">
+      <c r="A28" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C28" s="13" t="n">
         <v>0.15</v>
       </c>
+      <c r="D28" s="13" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="E28" s="12" t="n">
+        <f aca="false">IF($C$3=1,C28,D28)</f>
+        <v>0.03</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="C29" s="12" t="n">
+      <c r="A29" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C29" s="13" t="n">
         <v>1.5</v>
       </c>
+      <c r="D29" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="12" t="n">
+        <f aca="false">IF($C$3=1,C29,D29)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="3" t="s">
-        <v>29</v>
+      <c r="A30" s="5" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="4" t="s">
-        <v>30</v>
+      <c r="A31" s="3" t="s">
+        <v>34</v>
       </c>
       <c r="C31" s="9" t="n">
         <v>0.35</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="C32" s="13" t="n">
+      <c r="A32" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C32" s="14" t="n">
         <v>0.008</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="4" t="s">
-        <v>32</v>
+      <c r="A33" s="3" t="s">
+        <v>36</v>
       </c>
       <c r="C33" s="9" t="n">
         <v>0.15</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="4" t="s">
-        <v>33</v>
+      <c r="A34" s="3" t="s">
+        <v>37</v>
       </c>
       <c r="C34" s="9" t="n">
         <v>0.1</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="4" t="s">
-        <v>34</v>
+      <c r="A35" s="3" t="s">
+        <v>38</v>
       </c>
       <c r="C35" s="9" t="n">
         <v>0.5</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="3" t="s">
-        <v>35</v>
+      <c r="A36" s="5" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="4" t="s">
-        <v>36</v>
+      <c r="A37" s="3" t="s">
+        <v>40</v>
       </c>
       <c r="C37" s="8" t="n">
         <v>0.275</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="4" t="s">
-        <v>37</v>
+      <c r="A38" s="3" t="s">
+        <v>41</v>
       </c>
       <c r="C38" s="10" t="n">
         <v>0.1</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="4" t="s">
-        <v>38</v>
+      <c r="A39" s="3" t="s">
+        <v>42</v>
       </c>
       <c r="C39" s="10" t="n">
         <v>0.05</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="3" t="s">
-        <v>39</v>
+      <c r="A40" s="5" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="4" t="s">
+      <c r="A41" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C41" s="15" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C42" s="15" t="n">
+        <v>8500</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C43" s="15" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="5" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C46" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="D46" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="E46" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="F46" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="G46" s="16" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C47" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="D47" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E47" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F47" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" s="13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C48" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D48" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E48" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="F48" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G48" s="11" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C49" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D49" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E49" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F49" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="G49" s="11" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C50" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D50" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E50" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F50" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="G50" s="13" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C51" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D51" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E51" s="4" t="n">
         <v>40</v>
       </c>
-      <c r="C41" s="14" t="n">
+      <c r="F51" s="4" t="n">
         <v>150</v>
       </c>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="C42" s="14" t="n">
-        <v>8500</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="C43" s="14" t="n">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="3" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C46" s="15" t="s">
-        <v>44</v>
-      </c>
-      <c r="D46" s="15" t="s">
-        <v>45</v>
-      </c>
-      <c r="E46" s="15" t="s">
-        <v>46</v>
-      </c>
-      <c r="F46" s="15" t="s">
-        <v>47</v>
-      </c>
-      <c r="G46" s="15" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="C47" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="D47" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E47" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F47" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G47" s="12" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="C48" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D48" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E48" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="F48" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="G48" s="11" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="C49" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D49" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="E49" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="F49" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="G49" s="11" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="C50" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="D50" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E50" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F50" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="G50" s="12" t="n">
+      <c r="G51" s="4" t="n">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C52" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D52" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E52" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="F52" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="G52" s="13" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C53" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D53" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="E53" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="F53" s="15" t="n">
+        <v>12</v>
+      </c>
+      <c r="G53" s="15" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C54" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D54" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E54" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F54" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G54" s="13" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C55" s="13" t="n">
         <v>3</v>
       </c>
-    </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="C51" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D51" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E51" s="5" t="n">
-        <v>40</v>
-      </c>
-      <c r="F51" s="5" t="n">
-        <v>150</v>
-      </c>
-      <c r="G51" s="5" t="n">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="C52" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="D52" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E52" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="F52" s="12" t="n">
+      <c r="D55" s="13" t="n">
         <v>4</v>
       </c>
-      <c r="G52" s="12" t="n">
+      <c r="E55" s="13" t="n">
         <v>5</v>
       </c>
-    </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="C53" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D53" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="E53" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="F53" s="14" t="n">
-        <v>12</v>
-      </c>
-      <c r="G53" s="14" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="C54" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="D54" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E54" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F54" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="G54" s="12" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="C55" s="12" t="n">
+      <c r="F55" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="G55" s="13" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C56" s="13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D56" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E56" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="F56" s="13" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G56" s="13" t="n">
         <v>3</v>
       </c>
-      <c r="D55" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="E55" s="12" t="n">
-        <v>5</v>
-      </c>
-      <c r="F55" s="12" t="n">
-        <v>7</v>
-      </c>
-      <c r="G55" s="12" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="C56" s="12" t="n">
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C57" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D57" s="13" t="n">
         <v>0.5</v>
       </c>
-      <c r="D56" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E56" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="F56" s="12" t="n">
+      <c r="E57" s="13" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F57" s="13" t="n">
         <v>2.5</v>
       </c>
-      <c r="G56" s="12" t="n">
+      <c r="G57" s="13" t="n">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="C58" s="13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D58" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E58" s="13" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F58" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="G58" s="13" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="C57" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="D57" s="12" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E57" s="12" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="F57" s="12" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="G57" s="12" t="n">
-        <v>3.5</v>
-      </c>
-    </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="C58" s="12" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="D58" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="E58" s="12" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="F58" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="G58" s="12" t="n">
-        <v>3</v>
-      </c>
-    </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="4" t="s">
-        <v>61</v>
+      <c r="A59" s="3" t="s">
+        <v>65</v>
       </c>
       <c r="C59" s="9" t="n">
         <v>0.4</v>
@@ -1719,9 +1856,244 @@
         <v>1.3</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="2" t="s">
-        <v>62</v>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="5" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C63" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="D63" s="13" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E63" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="F63" s="13" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="G63" s="13" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="C64" s="13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D64" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E64" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F64" s="13" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G64" s="13" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C65" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D65" s="13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E65" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F65" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G65" s="13" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C66" s="13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D66" s="13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E66" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F66" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G66" s="13" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="C67" s="9" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D67" s="9" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E67" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F67" s="9" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="G67" s="9" t="n">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C70" s="12" t="n">
+        <f aca="false">IF($C$3=1,C55,C63)</f>
+        <v>2</v>
+      </c>
+      <c r="D70" s="12" t="n">
+        <f aca="false">IF($C$3=1,D55,D63)</f>
+        <v>2.5</v>
+      </c>
+      <c r="E70" s="12" t="n">
+        <f aca="false">IF($C$3=1,E55,E63)</f>
+        <v>3</v>
+      </c>
+      <c r="F70" s="12" t="n">
+        <f aca="false">IF($C$3=1,F55,F63)</f>
+        <v>3.5</v>
+      </c>
+      <c r="G70" s="12" t="n">
+        <f aca="false">IF($C$3=1,G55,G63)</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="C71" s="12" t="n">
+        <f aca="false">IF($C$3=1,C56,C64)</f>
+        <v>0.5</v>
+      </c>
+      <c r="D71" s="12" t="n">
+        <f aca="false">IF($C$3=1,D56,D64)</f>
+        <v>1</v>
+      </c>
+      <c r="E71" s="12" t="n">
+        <f aca="false">IF($C$3=1,E56,E64)</f>
+        <v>1</v>
+      </c>
+      <c r="F71" s="12" t="n">
+        <f aca="false">IF($C$3=1,F56,F64)</f>
+        <v>1.5</v>
+      </c>
+      <c r="G71" s="12" t="n">
+        <f aca="false">IF($C$3=1,G56,G64)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="C72" s="12" t="n">
+        <f aca="false">IF($C$3=1,C57,C65)</f>
+        <v>0</v>
+      </c>
+      <c r="D72" s="12" t="n">
+        <f aca="false">IF($C$3=1,D57,D65)</f>
+        <v>0.5</v>
+      </c>
+      <c r="E72" s="12" t="n">
+        <f aca="false">IF($C$3=1,E57,E65)</f>
+        <v>1</v>
+      </c>
+      <c r="F72" s="12" t="n">
+        <f aca="false">IF($C$3=1,F57,F65)</f>
+        <v>1</v>
+      </c>
+      <c r="G72" s="12" t="n">
+        <f aca="false">IF($C$3=1,G57,G65)</f>
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C73" s="12" t="n">
+        <f aca="false">IF($C$3=1,C58,C66)</f>
+        <v>0.5</v>
+      </c>
+      <c r="D73" s="12" t="n">
+        <f aca="false">IF($C$3=1,D58,D66)</f>
+        <v>0.5</v>
+      </c>
+      <c r="E73" s="12" t="n">
+        <f aca="false">IF($C$3=1,E58,E66)</f>
+        <v>1</v>
+      </c>
+      <c r="F73" s="12" t="n">
+        <f aca="false">IF($C$3=1,F58,F66)</f>
+        <v>1</v>
+      </c>
+      <c r="G73" s="12" t="n">
+        <f aca="false">IF($C$3=1,G58,G66)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C74" s="17" t="n">
+        <f aca="false">IF($C$3=1,C59,C67)</f>
+        <v>0.5</v>
+      </c>
+      <c r="D74" s="17" t="n">
+        <f aca="false">IF($C$3=1,D59,D67)</f>
+        <v>0.7</v>
+      </c>
+      <c r="E74" s="17" t="n">
+        <f aca="false">IF($C$3=1,E59,E67)</f>
+        <v>1</v>
+      </c>
+      <c r="F74" s="17" t="n">
+        <f aca="false">IF($C$3=1,F59,F67)</f>
+        <v>1.3</v>
+      </c>
+      <c r="G74" s="17" t="n">
+        <f aca="false">IF($C$3=1,G59,G67)</f>
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="2" t="s">
+        <v>78</v>
       </c>
     </row>
   </sheetData>
@@ -1741,7 +2113,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G47"/>
+  <dimension ref="A1:G49"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="58"/>
@@ -1750,370 +2122,370 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="str">
-        <f aca="false">"Active scenario: "&amp;INDEX({"Downside","Base","Upside"},Assumptions!$C$5)</f>
-        <v>Active scenario: Base</v>
+      <c r="A2" s="5" t="str">
+        <f aca="false">"Active scenario: "&amp;INDEX({"Downside","Base","Upside"},Assumptions!$C$5)&amp;" | Operating model: "&amp;INDEX({"Standard FDE team","Lean agent foundry"},Assumptions!$C$3)</f>
+        <v>Active scenario: Base | Operating model: Lean agent foundry</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C4" s="15" t="s">
-        <v>44</v>
-      </c>
-      <c r="D4" s="15" t="s">
-        <v>45</v>
-      </c>
-      <c r="E4" s="15" t="s">
-        <v>46</v>
-      </c>
-      <c r="F4" s="15" t="s">
-        <v>47</v>
-      </c>
-      <c r="G4" s="15" t="s">
+      <c r="C4" s="16" t="s">
         <v>48</v>
       </c>
+      <c r="D4" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="E4" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="F4" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="G4" s="16" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
-        <v>64</v>
+      <c r="A5" s="5" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="C6" s="16" t="n">
+      <c r="A6" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="C6" s="12" t="n">
         <f aca="false">Assumptions!C47</f>
         <v>2</v>
       </c>
-      <c r="D6" s="16" t="n">
+      <c r="D6" s="12" t="n">
         <f aca="false">Assumptions!D47</f>
         <v>0</v>
       </c>
-      <c r="E6" s="16" t="n">
+      <c r="E6" s="12" t="n">
         <f aca="false">Assumptions!E47</f>
         <v>0</v>
       </c>
-      <c r="F6" s="16" t="n">
+      <c r="F6" s="12" t="n">
         <f aca="false">Assumptions!F47</f>
         <v>0</v>
       </c>
-      <c r="G6" s="16" t="n">
+      <c r="G6" s="12" t="n">
         <f aca="false">Assumptions!G47</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="C7" s="16" t="n">
+      <c r="A7" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="C7" s="12" t="n">
         <f aca="false">Assumptions!C48*Assumptions!$C$9</f>
         <v>0</v>
       </c>
-      <c r="D7" s="16" t="n">
+      <c r="D7" s="12" t="n">
         <f aca="false">Assumptions!D48*Assumptions!$C$9</f>
         <v>1</v>
       </c>
-      <c r="E7" s="16" t="n">
+      <c r="E7" s="12" t="n">
         <f aca="false">Assumptions!E48*Assumptions!$C$9</f>
         <v>2</v>
       </c>
-      <c r="F7" s="16" t="n">
+      <c r="F7" s="12" t="n">
         <f aca="false">Assumptions!F48*Assumptions!$C$9</f>
         <v>1</v>
       </c>
-      <c r="G7" s="16" t="n">
+      <c r="G7" s="12" t="n">
         <f aca="false">Assumptions!G48*Assumptions!$C$9</f>
         <v>2</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="C8" s="16" t="n">
+      <c r="A8" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C8" s="12" t="n">
         <f aca="false">Assumptions!C49*Assumptions!$C$9</f>
         <v>0</v>
       </c>
-      <c r="D8" s="16" t="n">
+      <c r="D8" s="12" t="n">
         <f aca="false">Assumptions!D49*Assumptions!$C$9</f>
         <v>1</v>
       </c>
-      <c r="E8" s="16" t="n">
+      <c r="E8" s="12" t="n">
         <f aca="false">Assumptions!E49*Assumptions!$C$9</f>
         <v>1</v>
       </c>
-      <c r="F8" s="16" t="n">
+      <c r="F8" s="12" t="n">
         <f aca="false">Assumptions!F49*Assumptions!$C$9</f>
         <v>2</v>
       </c>
-      <c r="G8" s="16" t="n">
+      <c r="G8" s="12" t="n">
         <f aca="false">Assumptions!G49*Assumptions!$C$9</f>
         <v>2</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C9" s="16" t="n">
+      <c r="A9" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="C9" s="12" t="n">
         <f aca="false">C6</f>
         <v>2</v>
       </c>
-      <c r="D9" s="16" t="n">
+      <c r="D9" s="12" t="n">
         <f aca="false">C9+D6</f>
         <v>2</v>
       </c>
-      <c r="E9" s="16" t="n">
+      <c r="E9" s="12" t="n">
         <f aca="false">D9+E6</f>
         <v>2</v>
       </c>
-      <c r="F9" s="16" t="n">
+      <c r="F9" s="12" t="n">
         <f aca="false">E9+F6</f>
         <v>2</v>
       </c>
-      <c r="G9" s="16" t="n">
+      <c r="G9" s="12" t="n">
         <f aca="false">F9+G6</f>
         <v>2</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="C10" s="16" t="n">
+      <c r="A10" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="C10" s="12" t="n">
         <f aca="false">C7</f>
         <v>0</v>
       </c>
-      <c r="D10" s="16" t="n">
+      <c r="D10" s="12" t="n">
         <f aca="false">C10+D7</f>
         <v>1</v>
       </c>
-      <c r="E10" s="16" t="n">
+      <c r="E10" s="12" t="n">
         <f aca="false">D10+E7</f>
         <v>3</v>
       </c>
-      <c r="F10" s="16" t="n">
+      <c r="F10" s="12" t="n">
         <f aca="false">E10+F7</f>
         <v>4</v>
       </c>
-      <c r="G10" s="16" t="n">
+      <c r="G10" s="12" t="n">
         <f aca="false">F10+G7</f>
         <v>6</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="C11" s="16" t="n">
+      <c r="A11" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="C11" s="12" t="n">
         <f aca="false">C8</f>
         <v>0</v>
       </c>
-      <c r="D11" s="16" t="n">
+      <c r="D11" s="12" t="n">
         <f aca="false">C11+D8</f>
         <v>1</v>
       </c>
-      <c r="E11" s="16" t="n">
+      <c r="E11" s="12" t="n">
         <f aca="false">D11+E8</f>
         <v>2</v>
       </c>
-      <c r="F11" s="16" t="n">
+      <c r="F11" s="12" t="n">
         <f aca="false">E11+F8</f>
         <v>4</v>
       </c>
-      <c r="G11" s="16" t="n">
+      <c r="G11" s="12" t="n">
         <f aca="false">F11+G8</f>
         <v>6</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="C12" s="17" t="n">
+      <c r="A12" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="C12" s="18" t="n">
         <f aca="false">C9+C10+C11</f>
         <v>2</v>
       </c>
-      <c r="D12" s="17" t="n">
+      <c r="D12" s="18" t="n">
         <f aca="false">D9+D10+D11</f>
         <v>4</v>
       </c>
-      <c r="E12" s="17" t="n">
+      <c r="E12" s="18" t="n">
         <f aca="false">E9+E10+E11</f>
         <v>7</v>
       </c>
-      <c r="F12" s="17" t="n">
+      <c r="F12" s="18" t="n">
         <f aca="false">F9+F10+F11</f>
         <v>10</v>
       </c>
-      <c r="G12" s="17" t="n">
+      <c r="G12" s="18" t="n">
         <f aca="false">G9+G10+G11</f>
         <v>14</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="C13" s="18" t="n">
+      <c r="A13" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="C13" s="19" t="n">
         <f aca="false">IFERROR(C12/Assumptions!$C$41,0)</f>
         <v>0.0133333333333333</v>
       </c>
-      <c r="D13" s="18" t="n">
+      <c r="D13" s="19" t="n">
         <f aca="false">IFERROR(D12/Assumptions!$C$41,0)</f>
         <v>0.0266666666666667</v>
       </c>
-      <c r="E13" s="18" t="n">
+      <c r="E13" s="19" t="n">
         <f aca="false">IFERROR(E12/Assumptions!$C$41,0)</f>
         <v>0.0466666666666667</v>
       </c>
-      <c r="F13" s="18" t="n">
+      <c r="F13" s="19" t="n">
         <f aca="false">IFERROR(F12/Assumptions!$C$41,0)</f>
         <v>0.0666666666666667</v>
       </c>
-      <c r="G13" s="18" t="n">
+      <c r="G13" s="19" t="n">
         <f aca="false">IFERROR(G12/Assumptions!$C$41,0)</f>
         <v>0.0933333333333333</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
-        <v>73</v>
+      <c r="A14" s="5" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="C15" s="19" t="n">
+      <c r="A15" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C15" s="17" t="n">
         <f aca="false">C6*Assumptions!$C$13+C7*Assumptions!$C$11+C8*Assumptions!$C$12</f>
         <v>0.5</v>
       </c>
-      <c r="D15" s="19" t="n">
+      <c r="D15" s="17" t="n">
         <f aca="false">D6*Assumptions!$C$13+D7*Assumptions!$C$11+D8*Assumptions!$C$12</f>
         <v>1.15</v>
       </c>
-      <c r="E15" s="19" t="n">
+      <c r="E15" s="17" t="n">
         <f aca="false">E6*Assumptions!$C$13+E7*Assumptions!$C$11+E8*Assumptions!$C$12</f>
         <v>1.95</v>
       </c>
-      <c r="F15" s="19" t="n">
+      <c r="F15" s="17" t="n">
         <f aca="false">F6*Assumptions!$C$13+F7*Assumptions!$C$11+F8*Assumptions!$C$12</f>
         <v>1.5</v>
       </c>
-      <c r="G15" s="19" t="n">
+      <c r="G15" s="17" t="n">
         <f aca="false">G6*Assumptions!$C$13+G7*Assumptions!$C$11+G8*Assumptions!$C$12</f>
         <v>2.3</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="C16" s="19" t="n">
+      <c r="A16" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="C16" s="17" t="n">
         <f aca="false">Assumptions!$C$14*C15</f>
         <v>0.4</v>
       </c>
-      <c r="D16" s="19" t="n">
+      <c r="D16" s="17" t="n">
         <f aca="false">Assumptions!$C$14*D15+(1-Assumptions!$C$14)*C15</f>
         <v>1.02</v>
       </c>
-      <c r="E16" s="19" t="n">
+      <c r="E16" s="17" t="n">
         <f aca="false">Assumptions!$C$14*E15+(1-Assumptions!$C$14)*D15</f>
         <v>1.79</v>
       </c>
-      <c r="F16" s="19" t="n">
+      <c r="F16" s="17" t="n">
         <f aca="false">Assumptions!$C$14*F15+(1-Assumptions!$C$14)*E15</f>
         <v>1.59</v>
       </c>
-      <c r="G16" s="19" t="n">
+      <c r="G16" s="17" t="n">
         <f aca="false">Assumptions!$C$14*G15+(1-Assumptions!$C$14)*F15</f>
         <v>2.14</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="C17" s="19" t="n">
+      <c r="A17" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="C17" s="17" t="n">
         <f aca="false">C6*Assumptions!$C$17+C7*Assumptions!$C$15+C8*Assumptions!$C$16</f>
         <v>0.3</v>
       </c>
-      <c r="D17" s="19" t="n">
+      <c r="D17" s="17" t="n">
         <f aca="false">D6*Assumptions!$C$17+D7*Assumptions!$C$15+D8*Assumptions!$C$16</f>
         <v>0.4</v>
       </c>
-      <c r="E17" s="19" t="n">
+      <c r="E17" s="17" t="n">
         <f aca="false">E6*Assumptions!$C$17+E7*Assumptions!$C$15+E8*Assumptions!$C$16</f>
         <v>0.65</v>
       </c>
-      <c r="F17" s="19" t="n">
+      <c r="F17" s="17" t="n">
         <f aca="false">F6*Assumptions!$C$17+F7*Assumptions!$C$15+F8*Assumptions!$C$16</f>
         <v>0.55</v>
       </c>
-      <c r="G17" s="19" t="n">
+      <c r="G17" s="17" t="n">
         <f aca="false">G6*Assumptions!$C$17+G7*Assumptions!$C$15+G8*Assumptions!$C$16</f>
         <v>0.8</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="C18" s="19" t="n">
+      <c r="A18" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C18" s="17" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="D18" s="19" t="n">
+      <c r="D18" s="17" t="n">
         <f aca="false">C9*Assumptions!$C$19+C10*Assumptions!$C$11*Assumptions!$C$18+C11*Assumptions!$C$12*Assumptions!$C$18</f>
         <v>0.3</v>
       </c>
-      <c r="E18" s="19" t="n">
+      <c r="E18" s="17" t="n">
         <f aca="false">D9*Assumptions!$C$19+D10*Assumptions!$C$11*Assumptions!$C$18+D11*Assumptions!$C$12*Assumptions!$C$18</f>
         <v>0.53</v>
       </c>
-      <c r="F18" s="19" t="n">
+      <c r="F18" s="17" t="n">
         <f aca="false">E9*Assumptions!$C$19+E10*Assumptions!$C$11*Assumptions!$C$18+E11*Assumptions!$C$12*Assumptions!$C$18</f>
         <v>0.92</v>
       </c>
-      <c r="G18" s="19" t="n">
+      <c r="G18" s="17" t="n">
         <f aca="false">F9*Assumptions!$C$19+F10*Assumptions!$C$11*Assumptions!$C$18+F11*Assumptions!$C$12*Assumptions!$C$18</f>
         <v>1.22</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="C19" s="19" t="n">
+      <c r="A19" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C19" s="17" t="n">
         <f aca="false">0</f>
         <v>0</v>
       </c>
-      <c r="D19" s="19" t="n">
+      <c r="D19" s="17" t="n">
         <f aca="false">C9*Assumptions!$C$22+C10*Assumptions!$C$20+C11*Assumptions!$C$21</f>
         <v>0.3</v>
       </c>
-      <c r="E19" s="19" t="n">
+      <c r="E19" s="17" t="n">
         <f aca="false">D9*Assumptions!$C$22+D10*Assumptions!$C$20+D11*Assumptions!$C$21</f>
         <v>0.525</v>
       </c>
-      <c r="F19" s="19" t="n">
+      <c r="F19" s="17" t="n">
         <f aca="false">E9*Assumptions!$C$22+E10*Assumptions!$C$20+E11*Assumptions!$C$21</f>
         <v>0.9</v>
       </c>
-      <c r="G19" s="19" t="n">
+      <c r="G19" s="17" t="n">
         <f aca="false">F9*Assumptions!$C$22+F10*Assumptions!$C$20+F11*Assumptions!$C$21</f>
         <v>1.2</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="s">
-        <v>79</v>
+      <c r="A20" s="5" t="s">
+        <v>95</v>
       </c>
       <c r="C20" s="20" t="n">
         <f aca="false">SUM(C16:C19)</f>
@@ -2137,133 +2509,133 @@
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="C21" s="19" t="n">
+      <c r="A21" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="C21" s="17" t="n">
         <f aca="false">Assumptions!C50*Assumptions!$C$9*Assumptions!$C$31</f>
         <v>0</v>
       </c>
-      <c r="D21" s="19" t="n">
+      <c r="D21" s="17" t="n">
         <f aca="false">Assumptions!D50*Assumptions!$C$9*Assumptions!$C$31</f>
         <v>0</v>
       </c>
-      <c r="E21" s="19" t="n">
+      <c r="E21" s="17" t="n">
         <f aca="false">Assumptions!E50*Assumptions!$C$9*Assumptions!$C$31</f>
         <v>0.35</v>
       </c>
-      <c r="F21" s="19" t="n">
+      <c r="F21" s="17" t="n">
         <f aca="false">Assumptions!F50*Assumptions!$C$9*Assumptions!$C$31</f>
         <v>0.7</v>
       </c>
-      <c r="G21" s="19" t="n">
+      <c r="G21" s="17" t="n">
         <f aca="false">Assumptions!G50*Assumptions!$C$9*Assumptions!$C$31</f>
         <v>1.05</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="C22" s="19" t="n">
+      <c r="A22" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="C22" s="17" t="n">
         <f aca="false">Assumptions!C51*Assumptions!$C$9*Assumptions!$C$32</f>
         <v>0</v>
       </c>
-      <c r="D22" s="19" t="n">
+      <c r="D22" s="17" t="n">
         <f aca="false">Assumptions!D51*Assumptions!$C$9*Assumptions!$C$32</f>
         <v>0</v>
       </c>
-      <c r="E22" s="19" t="n">
+      <c r="E22" s="17" t="n">
         <f aca="false">Assumptions!E51*Assumptions!$C$9*Assumptions!$C$32</f>
         <v>0.32</v>
       </c>
-      <c r="F22" s="19" t="n">
+      <c r="F22" s="17" t="n">
         <f aca="false">Assumptions!F51*Assumptions!$C$9*Assumptions!$C$32</f>
         <v>1.2</v>
       </c>
-      <c r="G22" s="19" t="n">
+      <c r="G22" s="17" t="n">
         <f aca="false">Assumptions!G51*Assumptions!$C$9*Assumptions!$C$32</f>
         <v>3.2</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="C23" s="19" t="n">
+      <c r="A23" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="C23" s="17" t="n">
         <f aca="false">Assumptions!C52*Assumptions!$C$9*Assumptions!$C$33</f>
         <v>0</v>
       </c>
-      <c r="D23" s="19" t="n">
+      <c r="D23" s="17" t="n">
         <f aca="false">Assumptions!D52*Assumptions!$C$9*Assumptions!$C$33</f>
         <v>0.15</v>
       </c>
-      <c r="E23" s="19" t="n">
+      <c r="E23" s="17" t="n">
         <f aca="false">Assumptions!E52*Assumptions!$C$9*Assumptions!$C$33</f>
         <v>0.3</v>
       </c>
-      <c r="F23" s="19" t="n">
+      <c r="F23" s="17" t="n">
         <f aca="false">Assumptions!F52*Assumptions!$C$9*Assumptions!$C$33</f>
         <v>0.6</v>
       </c>
-      <c r="G23" s="19" t="n">
+      <c r="G23" s="17" t="n">
         <f aca="false">Assumptions!G52*Assumptions!$C$9*Assumptions!$C$33</f>
         <v>0.75</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="C24" s="19" t="n">
+      <c r="A24" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="C24" s="17" t="n">
         <f aca="false">Assumptions!C53*Assumptions!$C$9*Assumptions!$C$34</f>
         <v>0</v>
       </c>
-      <c r="D24" s="19" t="n">
+      <c r="D24" s="17" t="n">
         <f aca="false">Assumptions!D53*Assumptions!$C$9*Assumptions!$C$34</f>
         <v>0.2</v>
       </c>
-      <c r="E24" s="19" t="n">
+      <c r="E24" s="17" t="n">
         <f aca="false">Assumptions!E53*Assumptions!$C$9*Assumptions!$C$34</f>
         <v>0.6</v>
       </c>
-      <c r="F24" s="19" t="n">
+      <c r="F24" s="17" t="n">
         <f aca="false">Assumptions!F53*Assumptions!$C$9*Assumptions!$C$34</f>
         <v>1.2</v>
       </c>
-      <c r="G24" s="19" t="n">
+      <c r="G24" s="17" t="n">
         <f aca="false">Assumptions!G53*Assumptions!$C$9*Assumptions!$C$34</f>
         <v>2</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="C25" s="19" t="n">
+      <c r="A25" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C25" s="17" t="n">
         <f aca="false">Assumptions!C54*Assumptions!$C$9*Assumptions!$C$35</f>
         <v>0</v>
       </c>
-      <c r="D25" s="19" t="n">
+      <c r="D25" s="17" t="n">
         <f aca="false">Assumptions!D54*Assumptions!$C$9*Assumptions!$C$35</f>
         <v>0</v>
       </c>
-      <c r="E25" s="19" t="n">
+      <c r="E25" s="17" t="n">
         <f aca="false">Assumptions!E54*Assumptions!$C$9*Assumptions!$C$35</f>
         <v>0</v>
       </c>
-      <c r="F25" s="19" t="n">
+      <c r="F25" s="17" t="n">
         <f aca="false">Assumptions!F54*Assumptions!$C$9*Assumptions!$C$35</f>
         <v>0.5</v>
       </c>
-      <c r="G25" s="19" t="n">
+      <c r="G25" s="17" t="n">
         <f aca="false">Assumptions!G54*Assumptions!$C$9*Assumptions!$C$35</f>
         <v>1</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="3" t="s">
-        <v>85</v>
+      <c r="A26" s="5" t="s">
+        <v>101</v>
       </c>
       <c r="C26" s="20" t="n">
         <f aca="false">SUM(C21:C25)</f>
@@ -2287,8 +2659,8 @@
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="3" t="s">
-        <v>86</v>
+      <c r="A27" s="5" t="s">
+        <v>102</v>
       </c>
       <c r="C27" s="20" t="n">
         <f aca="false">C20+C26</f>
@@ -2312,447 +2684,477 @@
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="C28" s="19" t="n">
+      <c r="A28" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="C28" s="17" t="n">
         <f aca="false">C18+C21+C22+C23+C25</f>
         <v>0</v>
       </c>
-      <c r="D28" s="19" t="n">
+      <c r="D28" s="17" t="n">
         <f aca="false">D18+D21+D22+D23+D25</f>
         <v>0.45</v>
       </c>
-      <c r="E28" s="19" t="n">
+      <c r="E28" s="17" t="n">
         <f aca="false">E18+E21+E22+E23+E25</f>
         <v>1.5</v>
       </c>
-      <c r="F28" s="19" t="n">
+      <c r="F28" s="17" t="n">
         <f aca="false">F18+F21+F22+F23+F25</f>
         <v>3.92</v>
       </c>
-      <c r="G28" s="19" t="n">
+      <c r="G28" s="17" t="n">
         <f aca="false">G18+G21+G22+G23+G25</f>
         <v>7.22</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="C29" s="18" t="n">
+      <c r="A29" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="C29" s="19" t="n">
         <f aca="false">IFERROR(C28/C27,0)</f>
         <v>0</v>
       </c>
-      <c r="D29" s="18" t="n">
+      <c r="D29" s="19" t="n">
         <f aca="false">IFERROR(D28/D27,0)</f>
         <v>0.189873417721519</v>
       </c>
-      <c r="E29" s="18" t="n">
+      <c r="E29" s="19" t="n">
         <f aca="false">IFERROR(E28/E27,0)</f>
         <v>0.296150049358342</v>
       </c>
-      <c r="F29" s="18" t="n">
+      <c r="F29" s="19" t="n">
         <f aca="false">IFERROR(F28/F27,0)</f>
         <v>0.480392156862745</v>
       </c>
-      <c r="G29" s="18" t="n">
+      <c r="G29" s="19" t="n">
         <f aca="false">IFERROR(G28/G27,0)</f>
         <v>0.540419161676647</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="C30" s="18" t="n">
+      <c r="A30" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="C30" s="19" t="n">
         <f aca="false">IFERROR(C26/C27,0)</f>
         <v>0</v>
       </c>
-      <c r="D30" s="18" t="n">
+      <c r="D30" s="19" t="n">
         <f aca="false">IFERROR(D26/D27,0)</f>
         <v>0.147679324894515</v>
       </c>
-      <c r="E30" s="18" t="n">
+      <c r="E30" s="19" t="n">
         <f aca="false">IFERROR(E26/E27,0)</f>
         <v>0.309970384995064</v>
       </c>
-      <c r="F30" s="18" t="n">
+      <c r="F30" s="19" t="n">
         <f aca="false">IFERROR(F26/F27,0)</f>
         <v>0.514705882352941</v>
       </c>
-      <c r="G30" s="18" t="n">
+      <c r="G30" s="19" t="n">
         <f aca="false">IFERROR(G26/G27,0)</f>
         <v>0.598802395209581</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="C31" s="18" t="n">
+      <c r="A31" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="C31" s="19" t="n">
         <f aca="false">IFERROR(Assumptions!C51*Assumptions!$C$9/Assumptions!$C$42,0)</f>
         <v>0</v>
       </c>
-      <c r="D31" s="18" t="n">
+      <c r="D31" s="19" t="n">
         <f aca="false">IFERROR(Assumptions!D51*Assumptions!$C$9/Assumptions!$C$42,0)</f>
         <v>0</v>
       </c>
-      <c r="E31" s="18" t="n">
+      <c r="E31" s="19" t="n">
         <f aca="false">IFERROR(Assumptions!E51*Assumptions!$C$9/Assumptions!$C$42,0)</f>
         <v>0.00470588235294118</v>
       </c>
-      <c r="F31" s="18" t="n">
+      <c r="F31" s="19" t="n">
         <f aca="false">IFERROR(Assumptions!F51*Assumptions!$C$9/Assumptions!$C$42,0)</f>
         <v>0.0176470588235294</v>
       </c>
-      <c r="G31" s="18" t="n">
+      <c r="G31" s="19" t="n">
         <f aca="false">IFERROR(Assumptions!G51*Assumptions!$C$9/Assumptions!$C$42,0)</f>
         <v>0.0470588235294118</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="3" t="s">
-        <v>91</v>
+      <c r="A32" s="5" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="C33" s="16" t="n">
-        <f aca="false">MAX(Assumptions!$C$29,C6*Assumptions!$C$26+C7*Assumptions!$C$24+C8*Assumptions!$C$25)</f>
+      <c r="A33" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="C33" s="12" t="n">
+        <f aca="false">MAX(Assumptions!$E$29,C6*Assumptions!$E$26+C7*Assumptions!$E$24+C8*Assumptions!$E$25)</f>
+        <v>1</v>
+      </c>
+      <c r="D33" s="12" t="n">
+        <f aca="false">MAX(Assumptions!$E$29,D6*Assumptions!$E$26+D7*Assumptions!$E$24+D8*Assumptions!$E$25+(C9+C10)*Assumptions!$E$27+C11*Assumptions!$E$28)</f>
+        <v>1</v>
+      </c>
+      <c r="E33" s="12" t="n">
+        <f aca="false">MAX(Assumptions!$E$29,E6*Assumptions!$E$26+E7*Assumptions!$E$24+E8*Assumptions!$E$25+(D9+D10)*Assumptions!$E$27+D11*Assumptions!$E$28)</f>
+        <v>1</v>
+      </c>
+      <c r="F33" s="12" t="n">
+        <f aca="false">MAX(Assumptions!$E$29,F6*Assumptions!$E$26+F7*Assumptions!$E$24+F8*Assumptions!$E$25+(E9+E10)*Assumptions!$E$27+E11*Assumptions!$E$28)</f>
+        <v>1</v>
+      </c>
+      <c r="G33" s="12" t="n">
+        <f aca="false">MAX(Assumptions!$E$29,G6*Assumptions!$E$26+G7*Assumptions!$E$24+G8*Assumptions!$E$25+(F9+F10)*Assumptions!$E$27+F11*Assumptions!$E$28)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="C34" s="12" t="n">
+        <f aca="false">Assumptions!C70</f>
+        <v>2</v>
+      </c>
+      <c r="D34" s="12" t="n">
+        <f aca="false">Assumptions!D70</f>
+        <v>2.5</v>
+      </c>
+      <c r="E34" s="12" t="n">
+        <f aca="false">Assumptions!E70</f>
+        <v>3</v>
+      </c>
+      <c r="F34" s="12" t="n">
+        <f aca="false">Assumptions!F70</f>
+        <v>3.5</v>
+      </c>
+      <c r="G34" s="12" t="n">
+        <f aca="false">Assumptions!G70</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="C35" s="12" t="n">
+        <f aca="false">Assumptions!C71</f>
+        <v>0.5</v>
+      </c>
+      <c r="D35" s="12" t="n">
+        <f aca="false">Assumptions!D71</f>
+        <v>1</v>
+      </c>
+      <c r="E35" s="12" t="n">
+        <f aca="false">Assumptions!E71</f>
+        <v>1</v>
+      </c>
+      <c r="F35" s="12" t="n">
+        <f aca="false">Assumptions!F71</f>
         <v>1.5</v>
       </c>
-      <c r="D33" s="16" t="n">
-        <f aca="false">MAX(Assumptions!$C$29,D6*Assumptions!$C$26+D7*Assumptions!$C$24+D8*Assumptions!$C$25+(C9+C10)*Assumptions!$C$27+C11*Assumptions!$C$28)</f>
+      <c r="G35" s="12" t="n">
+        <f aca="false">Assumptions!G71</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="C36" s="12" t="n">
+        <f aca="false">Assumptions!C72</f>
+        <v>0</v>
+      </c>
+      <c r="D36" s="12" t="n">
+        <f aca="false">Assumptions!D72</f>
+        <v>0.5</v>
+      </c>
+      <c r="E36" s="12" t="n">
+        <f aca="false">Assumptions!E72</f>
+        <v>1</v>
+      </c>
+      <c r="F36" s="12" t="n">
+        <f aca="false">Assumptions!F72</f>
+        <v>1</v>
+      </c>
+      <c r="G36" s="12" t="n">
+        <f aca="false">Assumptions!G72</f>
         <v>1.5</v>
       </c>
-      <c r="E33" s="16" t="n">
-        <f aca="false">MAX(Assumptions!$C$29,E6*Assumptions!$C$26+E7*Assumptions!$C$24+E8*Assumptions!$C$25+(D9+D10)*Assumptions!$C$27+D11*Assumptions!$C$28)</f>
-        <v>1.75</v>
-      </c>
-      <c r="F33" s="16" t="n">
-        <f aca="false">MAX(Assumptions!$C$29,F6*Assumptions!$C$26+F7*Assumptions!$C$24+F8*Assumptions!$C$25+(E9+E10)*Assumptions!$C$27+E11*Assumptions!$C$28)</f>
-        <v>2.35</v>
-      </c>
-      <c r="G33" s="16" t="n">
-        <f aca="false">MAX(Assumptions!$C$29,G6*Assumptions!$C$26+G7*Assumptions!$C$24+G8*Assumptions!$C$25+(F9+F10)*Assumptions!$C$27+F11*Assumptions!$C$28)</f>
-        <v>3.2</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="C34" s="16" t="n">
-        <f aca="false">Assumptions!C55</f>
-        <v>3</v>
-      </c>
-      <c r="D34" s="16" t="n">
-        <f aca="false">Assumptions!D55</f>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="C37" s="12" t="n">
+        <f aca="false">Assumptions!C73</f>
+        <v>0.5</v>
+      </c>
+      <c r="D37" s="12" t="n">
+        <f aca="false">Assumptions!D73</f>
+        <v>0.5</v>
+      </c>
+      <c r="E37" s="12" t="n">
+        <f aca="false">Assumptions!E73</f>
+        <v>1</v>
+      </c>
+      <c r="F37" s="12" t="n">
+        <f aca="false">Assumptions!F73</f>
+        <v>1</v>
+      </c>
+      <c r="G37" s="12" t="n">
+        <f aca="false">Assumptions!G73</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="C38" s="18" t="n">
+        <f aca="false">SUM(C33:C37)</f>
         <v>4</v>
       </c>
-      <c r="E34" s="16" t="n">
-        <f aca="false">Assumptions!E55</f>
-        <v>5</v>
-      </c>
-      <c r="F34" s="16" t="n">
-        <f aca="false">Assumptions!F55</f>
+      <c r="D38" s="18" t="n">
+        <f aca="false">SUM(D33:D37)</f>
+        <v>5.5</v>
+      </c>
+      <c r="E38" s="18" t="n">
+        <f aca="false">SUM(E33:E37)</f>
         <v>7</v>
       </c>
-      <c r="G34" s="16" t="n">
-        <f aca="false">Assumptions!G55</f>
-        <v>9</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="C35" s="16" t="n">
-        <f aca="false">Assumptions!C56</f>
+      <c r="F38" s="18" t="n">
+        <f aca="false">SUM(F33:F37)</f>
+        <v>8</v>
+      </c>
+      <c r="G38" s="18" t="n">
+        <f aca="false">SUM(G33:G37)</f>
+        <v>9.5</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="5" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C40" s="17" t="n">
+        <f aca="false">C38*Assumptions!$C$37</f>
+        <v>1.1</v>
+      </c>
+      <c r="D40" s="17" t="n">
+        <f aca="false">D38*Assumptions!$C$37</f>
+        <v>1.5125</v>
+      </c>
+      <c r="E40" s="17" t="n">
+        <f aca="false">E38*Assumptions!$C$37</f>
+        <v>1.925</v>
+      </c>
+      <c r="F40" s="17" t="n">
+        <f aca="false">F38*Assumptions!$C$37</f>
+        <v>2.2</v>
+      </c>
+      <c r="G40" s="17" t="n">
+        <f aca="false">G38*Assumptions!$C$37</f>
+        <v>2.6125</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="C41" s="17" t="n">
+        <f aca="false">Assumptions!C74</f>
         <v>0.5</v>
       </c>
-      <c r="D35" s="16" t="n">
-        <f aca="false">Assumptions!D56</f>
-        <v>1</v>
-      </c>
-      <c r="E35" s="16" t="n">
-        <f aca="false">Assumptions!E56</f>
-        <v>2</v>
-      </c>
-      <c r="F35" s="16" t="n">
-        <f aca="false">Assumptions!F56</f>
-        <v>2.5</v>
-      </c>
-      <c r="G35" s="16" t="n">
-        <f aca="false">Assumptions!G56</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="C36" s="16" t="n">
-        <f aca="false">Assumptions!C57</f>
-        <v>0</v>
-      </c>
-      <c r="D36" s="16" t="n">
-        <f aca="false">Assumptions!D57</f>
-        <v>0.5</v>
-      </c>
-      <c r="E36" s="16" t="n">
-        <f aca="false">Assumptions!E57</f>
-        <v>1.5</v>
-      </c>
-      <c r="F36" s="16" t="n">
-        <f aca="false">Assumptions!F57</f>
-        <v>2.5</v>
-      </c>
-      <c r="G36" s="16" t="n">
-        <f aca="false">Assumptions!G57</f>
-        <v>3.5</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="C37" s="16" t="n">
-        <f aca="false">Assumptions!C58</f>
-        <v>0.5</v>
-      </c>
-      <c r="D37" s="16" t="n">
-        <f aca="false">Assumptions!D58</f>
-        <v>1</v>
-      </c>
-      <c r="E37" s="16" t="n">
-        <f aca="false">Assumptions!E58</f>
-        <v>1.5</v>
-      </c>
-      <c r="F37" s="16" t="n">
-        <f aca="false">Assumptions!F58</f>
-        <v>2</v>
-      </c>
-      <c r="G37" s="16" t="n">
-        <f aca="false">Assumptions!G58</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="C38" s="17" t="n">
-        <f aca="false">SUM(C33:C37)</f>
-        <v>5.5</v>
-      </c>
-      <c r="D38" s="17" t="n">
-        <f aca="false">SUM(D33:D37)</f>
-        <v>8</v>
-      </c>
-      <c r="E38" s="17" t="n">
-        <f aca="false">SUM(E33:E37)</f>
-        <v>11.75</v>
-      </c>
-      <c r="F38" s="17" t="n">
-        <f aca="false">SUM(F33:F37)</f>
-        <v>16.35</v>
-      </c>
-      <c r="G38" s="17" t="n">
-        <f aca="false">SUM(G33:G37)</f>
-        <v>21.7</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="3" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="C40" s="19" t="n">
-        <f aca="false">C38*Assumptions!$C$37</f>
-        <v>1.5125</v>
-      </c>
-      <c r="D40" s="19" t="n">
-        <f aca="false">D38*Assumptions!$C$37</f>
-        <v>2.2</v>
-      </c>
-      <c r="E40" s="19" t="n">
-        <f aca="false">E38*Assumptions!$C$37</f>
-        <v>3.23125</v>
-      </c>
-      <c r="F40" s="19" t="n">
-        <f aca="false">F38*Assumptions!$C$37</f>
-        <v>4.49625</v>
-      </c>
-      <c r="G40" s="19" t="n">
-        <f aca="false">G38*Assumptions!$C$37</f>
-        <v>5.9675</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="C41" s="19" t="n">
-        <f aca="false">Assumptions!C59</f>
-        <v>0.4</v>
-      </c>
-      <c r="D41" s="19" t="n">
-        <f aca="false">Assumptions!D59</f>
-        <v>0.55</v>
-      </c>
-      <c r="E41" s="19" t="n">
-        <f aca="false">Assumptions!E59</f>
-        <v>0.8</v>
-      </c>
-      <c r="F41" s="19" t="n">
-        <f aca="false">Assumptions!F59</f>
-        <v>1</v>
-      </c>
-      <c r="G41" s="19" t="n">
-        <f aca="false">Assumptions!G59</f>
+      <c r="D41" s="17" t="n">
+        <f aca="false">Assumptions!D74</f>
+        <v>0.7</v>
+      </c>
+      <c r="E41" s="17" t="n">
+        <f aca="false">Assumptions!E74</f>
+        <v>1</v>
+      </c>
+      <c r="F41" s="17" t="n">
+        <f aca="false">Assumptions!F74</f>
         <v>1.3</v>
       </c>
+      <c r="G41" s="17" t="n">
+        <f aca="false">Assumptions!G74</f>
+        <v>1.6</v>
+      </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="C42" s="19" t="n">
+      <c r="A42" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="C42" s="17" t="n">
         <f aca="false">C15*Assumptions!$C$38+C26*Assumptions!$C$39</f>
         <v>0.05</v>
       </c>
-      <c r="D42" s="19" t="n">
+      <c r="D42" s="17" t="n">
         <f aca="false">D15*Assumptions!$C$38+D26*Assumptions!$C$39</f>
         <v>0.1325</v>
       </c>
-      <c r="E42" s="19" t="n">
+      <c r="E42" s="17" t="n">
         <f aca="false">E15*Assumptions!$C$38+E26*Assumptions!$C$39</f>
         <v>0.2735</v>
       </c>
-      <c r="F42" s="19" t="n">
+      <c r="F42" s="17" t="n">
         <f aca="false">F15*Assumptions!$C$38+F26*Assumptions!$C$39</f>
         <v>0.36</v>
       </c>
-      <c r="G42" s="19" t="n">
+      <c r="G42" s="17" t="n">
         <f aca="false">G15*Assumptions!$C$38+G26*Assumptions!$C$39</f>
         <v>0.63</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="3" t="s">
-        <v>102</v>
+      <c r="A43" s="5" t="s">
+        <v>118</v>
       </c>
       <c r="C43" s="20" t="n">
         <f aca="false">SUM(C40:C42)</f>
-        <v>1.9625</v>
+        <v>1.65</v>
       </c>
       <c r="D43" s="20" t="n">
         <f aca="false">SUM(D40:D42)</f>
-        <v>2.8825</v>
+        <v>2.345</v>
       </c>
       <c r="E43" s="20" t="n">
         <f aca="false">SUM(E40:E42)</f>
-        <v>4.30475</v>
+        <v>3.1985</v>
       </c>
       <c r="F43" s="20" t="n">
         <f aca="false">SUM(F40:F42)</f>
-        <v>5.85625</v>
+        <v>3.86</v>
       </c>
       <c r="G43" s="20" t="n">
         <f aca="false">SUM(G40:G42)</f>
-        <v>7.8975</v>
+        <v>4.8425</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="3" t="s">
-        <v>103</v>
+      <c r="A44" s="5" t="s">
+        <v>119</v>
       </c>
       <c r="C44" s="20" t="n">
         <f aca="false">C27-C43</f>
-        <v>-1.2625</v>
+        <v>-0.95</v>
       </c>
       <c r="D44" s="20" t="n">
         <f aca="false">D27-D43</f>
-        <v>-0.5125</v>
+        <v>0.0249999999999999</v>
       </c>
       <c r="E44" s="20" t="n">
         <f aca="false">E27-E43</f>
-        <v>0.76025</v>
+        <v>1.8665</v>
       </c>
       <c r="F44" s="20" t="n">
         <f aca="false">F27-F43</f>
-        <v>2.30375</v>
+        <v>4.3</v>
       </c>
       <c r="G44" s="20" t="n">
         <f aca="false">G27-G43</f>
-        <v>5.4625</v>
+        <v>8.5175</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="C45" s="18" t="n">
+      <c r="A45" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="C45" s="19" t="n">
         <f aca="false">IFERROR(C44/C27,0)</f>
-        <v>-1.80357142857143</v>
-      </c>
-      <c r="D45" s="18" t="n">
+        <v>-1.35714285714286</v>
+      </c>
+      <c r="D45" s="19" t="n">
         <f aca="false">IFERROR(D44/D27,0)</f>
-        <v>-0.216244725738397</v>
-      </c>
-      <c r="E45" s="18" t="n">
+        <v>0.010548523206751</v>
+      </c>
+      <c r="E45" s="19" t="n">
         <f aca="false">IFERROR(E44/E27,0)</f>
-        <v>0.150098716683119</v>
-      </c>
-      <c r="F45" s="18" t="n">
+        <v>0.368509378084896</v>
+      </c>
+      <c r="F45" s="19" t="n">
         <f aca="false">IFERROR(F44/F27,0)</f>
-        <v>0.282322303921569</v>
-      </c>
-      <c r="G45" s="18" t="n">
+        <v>0.526960784313726</v>
+      </c>
+      <c r="G45" s="19" t="n">
         <f aca="false">IFERROR(G44/G27,0)</f>
-        <v>0.408869760479042</v>
+        <v>0.637537425149701</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="C46" s="19" t="n">
+      <c r="A46" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="C46" s="17" t="n">
         <f aca="false">C44</f>
-        <v>-1.2625</v>
-      </c>
-      <c r="D46" s="19" t="n">
+        <v>-0.95</v>
+      </c>
+      <c r="D46" s="17" t="n">
         <f aca="false">C46+D44</f>
-        <v>-1.775</v>
-      </c>
-      <c r="E46" s="19" t="n">
+        <v>-0.925</v>
+      </c>
+      <c r="E46" s="17" t="n">
         <f aca="false">D46+E44</f>
-        <v>-1.01475</v>
-      </c>
-      <c r="F46" s="19" t="n">
+        <v>0.9415</v>
+      </c>
+      <c r="F46" s="17" t="n">
         <f aca="false">E46+F44</f>
-        <v>1.289</v>
-      </c>
-      <c r="G46" s="19" t="n">
+        <v>5.2415</v>
+      </c>
+      <c r="G46" s="17" t="n">
         <f aca="false">F46+G44</f>
-        <v>6.7515</v>
+        <v>13.759</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="3" t="s">
-        <v>106</v>
+      <c r="A47" s="5" t="s">
+        <v>122</v>
       </c>
       <c r="C47" s="20" t="n">
         <f aca="false">-MIN(0,MIN(C46:G46))</f>
-        <v>1.775</v>
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="C48" s="12" t="n">
+        <f aca="false">IFERROR((C6+C7+C8)/C33,0)</f>
+        <v>2</v>
+      </c>
+      <c r="D48" s="12" t="n">
+        <f aca="false">IFERROR((D6+D7+D8)/D33,0)</f>
+        <v>2</v>
+      </c>
+      <c r="E48" s="12" t="n">
+        <f aca="false">IFERROR((E6+E7+E8)/E33,0)</f>
+        <v>3</v>
+      </c>
+      <c r="F48" s="12" t="n">
+        <f aca="false">IFERROR((F6+F7+F8)/F33,0)</f>
+        <v>3</v>
+      </c>
+      <c r="G48" s="12" t="n">
+        <f aca="false">IFERROR((G6+G7+G8)/G33,0)</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="2" t="s">
+        <v>124</v>
       </c>
     </row>
   </sheetData>
@@ -2780,28 +3182,28 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>107</v>
+        <v>125</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>108</v>
+        <v>126</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C4" s="15" t="s">
-        <v>109</v>
-      </c>
-      <c r="D4" s="15" t="s">
-        <v>110</v>
-      </c>
-      <c r="E4" s="15" t="s">
-        <v>111</v>
+      <c r="C4" s="16" t="s">
+        <v>127</v>
+      </c>
+      <c r="D4" s="16" t="s">
+        <v>128</v>
+      </c>
+      <c r="E4" s="16" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
-        <v>112</v>
+      <c r="A5" s="3" t="s">
+        <v>130</v>
       </c>
       <c r="C5" s="21" t="n">
         <v>4</v>
@@ -2814,8 +3216,8 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
-        <v>113</v>
+      <c r="A6" s="3" t="s">
+        <v>131</v>
       </c>
       <c r="C6" s="21" t="n">
         <v>1</v>
@@ -2828,8 +3230,8 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
-        <v>114</v>
+      <c r="A7" s="3" t="s">
+        <v>132</v>
       </c>
       <c r="C7" s="21" t="n">
         <v>10</v>
@@ -2842,13 +3244,13 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
-        <v>115</v>
+      <c r="A9" s="5" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
-        <v>116</v>
+      <c r="A10" s="3" t="s">
+        <v>134</v>
       </c>
       <c r="C10" s="22" t="n">
         <f aca="false">Model!G27</f>
@@ -2856,8 +3258,8 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
-        <v>117</v>
+      <c r="A11" s="3" t="s">
+        <v>135</v>
       </c>
       <c r="C11" s="22" t="n">
         <f aca="false">Model!G28</f>
@@ -2865,214 +3267,214 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="C12" s="19" t="n">
+      <c r="A12" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="C12" s="17" t="n">
         <f aca="false">C10-C11</f>
         <v>6.14</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
-        <v>119</v>
+      <c r="A13" s="3" t="s">
+        <v>137</v>
       </c>
       <c r="C13" s="22" t="n">
         <f aca="false">Model!G44</f>
-        <v>5.4625</v>
+        <v>8.5175</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="C15" s="15" t="s">
-        <v>109</v>
-      </c>
-      <c r="D15" s="15" t="s">
-        <v>110</v>
-      </c>
-      <c r="E15" s="15" t="s">
-        <v>111</v>
+      <c r="A15" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="C15" s="16" t="s">
+        <v>127</v>
+      </c>
+      <c r="D15" s="16" t="s">
+        <v>128</v>
+      </c>
+      <c r="E15" s="16" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="C16" s="19" t="n">
+      <c r="A16" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="C16" s="17" t="n">
         <f aca="false">$C$11*C5+$C$12*C6</f>
         <v>35.02</v>
       </c>
-      <c r="D16" s="19" t="n">
+      <c r="D16" s="17" t="n">
         <f aca="false">$C$11*D5+$C$12*D6</f>
         <v>52.53</v>
       </c>
-      <c r="E16" s="19" t="n">
+      <c r="E16" s="17" t="n">
         <f aca="false">$C$11*E5+$C$12*E6</f>
         <v>70.04</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="C17" s="19" t="n">
+      <c r="A17" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="C17" s="17" t="n">
         <f aca="false">MAX(0,$C$13)*C7</f>
-        <v>54.625</v>
-      </c>
-      <c r="D17" s="19" t="n">
+        <v>85.175</v>
+      </c>
+      <c r="D17" s="17" t="n">
         <f aca="false">MAX(0,$C$13)*D7</f>
-        <v>81.9375</v>
-      </c>
-      <c r="E17" s="19" t="n">
+        <v>127.7625</v>
+      </c>
+      <c r="E17" s="17" t="n">
         <f aca="false">MAX(0,$C$13)*E7</f>
-        <v>109.25</v>
+        <v>170.35</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="s">
-        <v>123</v>
+      <c r="A18" s="3" t="s">
+        <v>141</v>
       </c>
       <c r="C18" s="20" t="n">
         <f aca="false">AVERAGE(C16:C17)</f>
-        <v>44.8225</v>
+        <v>60.0975</v>
       </c>
       <c r="D18" s="20" t="n">
         <f aca="false">AVERAGE(D16:D17)</f>
-        <v>67.23375</v>
+        <v>90.14625</v>
       </c>
       <c r="E18" s="20" t="n">
         <f aca="false">AVERAGE(E16:E17)</f>
-        <v>89.645</v>
+        <v>120.195</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="s">
-        <v>124</v>
+      <c r="A19" s="3" t="s">
+        <v>142</v>
       </c>
       <c r="C19" s="7" t="n">
         <f aca="false">IFERROR(C18/$C$10,0)</f>
-        <v>3.35497754491018</v>
+        <v>4.49831586826347</v>
       </c>
       <c r="D19" s="7" t="n">
         <f aca="false">IFERROR(D18/$C$10,0)</f>
-        <v>5.03246631736527</v>
+        <v>6.74747380239521</v>
       </c>
       <c r="E19" s="7" t="n">
         <f aca="false">IFERROR(E18/$C$10,0)</f>
-        <v>6.70995508982036</v>
+        <v>8.99663173652695</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3" t="s">
-        <v>125</v>
+      <c r="A21" s="5" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="s">
-        <v>126</v>
+      <c r="A22" s="3" t="s">
+        <v>144</v>
       </c>
       <c r="C22" s="21" t="n">
         <v>20</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="4" t="s">
-        <v>127</v>
+      <c r="A23" s="3" t="s">
+        <v>145</v>
       </c>
       <c r="C23" s="21" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4" t="s">
-        <v>128</v>
+      <c r="A24" s="3" t="s">
+        <v>146</v>
       </c>
       <c r="C24" s="10" t="n">
         <v>0.15</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C26" s="15" t="s">
-        <v>109</v>
-      </c>
-      <c r="D26" s="15" t="s">
-        <v>110</v>
-      </c>
-      <c r="E26" s="15" t="s">
-        <v>111</v>
+      <c r="C26" s="16" t="s">
+        <v>127</v>
+      </c>
+      <c r="D26" s="16" t="s">
+        <v>128</v>
+      </c>
+      <c r="E26" s="16" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="C27" s="19" t="n">
+      <c r="A27" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="C27" s="17" t="n">
         <f aca="false">C18*(1-$C$24)/$C$22</f>
-        <v>1.90495625</v>
-      </c>
-      <c r="D27" s="19" t="n">
+        <v>2.55414375</v>
+      </c>
+      <c r="D27" s="17" t="n">
         <f aca="false">D18*(1-$C$24)/$C$22</f>
-        <v>2.857434375</v>
-      </c>
-      <c r="E27" s="19" t="n">
+        <v>3.831215625</v>
+      </c>
+      <c r="E27" s="17" t="n">
         <f aca="false">E18*(1-$C$24)/$C$22</f>
-        <v>3.8099125</v>
+        <v>5.1082875</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="C28" s="19" t="n">
+      <c r="A28" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="C28" s="17" t="n">
         <f aca="false">C18*(1-$C$24)/$C$23</f>
-        <v>3.8099125</v>
-      </c>
-      <c r="D28" s="19" t="n">
+        <v>5.1082875</v>
+      </c>
+      <c r="D28" s="17" t="n">
         <f aca="false">D18*(1-$C$24)/$C$23</f>
-        <v>5.71486875</v>
-      </c>
-      <c r="E28" s="19" t="n">
+        <v>7.66243125</v>
+      </c>
+      <c r="E28" s="17" t="n">
         <f aca="false">E18*(1-$C$24)/$C$23</f>
-        <v>7.619825</v>
+        <v>10.216575</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="3" t="s">
-        <v>131</v>
+      <c r="A30" s="5" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="C31" s="4" t="s">
-        <v>133</v>
+      <c r="A31" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="C32" s="4" t="s">
-        <v>135</v>
+      <c r="A32" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="4" t="s">
-        <v>136</v>
-      </c>
-      <c r="C33" s="4" t="s">
-        <v>137</v>
+      <c r="A33" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="C34" s="4" t="s">
-        <v>139</v>
+      <c r="A34" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>157</v>
       </c>
     </row>
   </sheetData>

</xml_diff>